<commit_message>
chore: DOI-stamped rebuild (10.5281/zenodo.21333712)
</commit_message>
<xml_diff>
--- a/sa-ecommerce-import-trends-2026-jlog.xlsx
+++ b/sa-ecommerce-import-trends-2026-jlog.xlsx
@@ -63,7 +63,7 @@
     </font>
     <font>
       <name val="Arial"/>
-      <color rgb="005A6B62"/>
+      <color rgb="001C5636"/>
       <sz val="11"/>
     </font>
     <font>
@@ -605,7 +605,7 @@
     <row r="19">
       <c r="B19" s="7" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>10.5281/zenodo.21333712</t>
         </is>
       </c>
     </row>
@@ -619,7 +619,7 @@
     <row r="22">
       <c r="B22" s="6" t="inlineStr">
         <is>
-          <t>JLog (JetLog (Pty) Ltd). "South Africa E-Commerce Import Trends", version 1.0, 2026. Derived from SARS Trade Statistics. CC BY 4.0. https://jlog.co.za/research/sa-ecommerce-import-trends/</t>
+          <t>JLog (JetLog (Pty) Ltd). "South Africa E-Commerce Import Trends", version 1.0, 2026. Derived from SARS Trade Statistics. CC BY 4.0. https://jlog.co.za/research/sa-ecommerce-import-trends/ doi:10.5281/zenodo.21333712</t>
         </is>
       </c>
     </row>

</xml_diff>